<commit_message>
test(m3): add sprint 1 unit test evidence
3 tests pass for TopicStatusService: publish unpublished topic,
reject already-published topic, reject wrong teacher ownership.
All 23 project tests pass (0 failures).
</commit_message>
<xml_diff>
--- a/test-evidence/M3-Cao-Yuhan/UT-M3-table.xlsx
+++ b/test-evidence/M3-Cao-Yuhan/UT-M3-table.xlsx
@@ -2,36 +2,194 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="20752" windowHeight="9555" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Tests" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="23">
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -40,16 +198,210 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -58,36 +410,513 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FFB2B2B2"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FFB2B2B2"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FFB2B2B2"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <dxfs count="7">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF08090C"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.8"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF08090C"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.8"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+  </dxfs>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="中色系标题行镶边行表格样式_6e22f3" count="7">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    </tableStyle>
+  </tableStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -438,7 +1267,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -448,168 +1276,272 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="17.5663716814159" customWidth="1" min="1" max="1"/>
+    <col width="11.7256637168142" customWidth="1" min="2" max="2"/>
+    <col width="50.3805309734513" customWidth="1" min="3" max="7"/>
+    <col width="16.3185840707965" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="22.5" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Test Name/ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Precondition (if any)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Output</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Expected</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Test process</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="65" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>UT-M3-S1-01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>ProjectTopicRepository and TopicStatusServiceImpl under test; topic (id=10) is unpublished, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>publishTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Returns ProjectTopic with status = available.</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Topic status changes to available when published by owner.</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Returned topic has status = available as asserted by assertEquals.</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="52" customHeight="1">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>UT-M3-S1-02</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Topic (id=10) is already in available status, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>publishTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Throws IllegalStateException with message "Only unpublished topics can be published".</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>Already-published topic cannot be published again; exception message is clear.</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>IllegalStateException thrown with expected message as asserted by assertThrows.</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="4" ht="73" customHeight="1">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>UT-M3-S1-03</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Topic (id=10) belongs to teacher (id=1), not teacher (id=99).</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>publishTopic(topicId=10, teacherId=99)</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Throws IllegalArgumentException with message "Topic not found or access denied".</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Topic not found or access denied for wrong teacher; ownership enforced.</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>IllegalArgumentException thrown with expected message as asserted by assertThrows.</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="67" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>UT-M3-S2-01</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="C5" s="10" t="inlineStr"/>
+      <c r="D5" s="10" t="inlineStr"/>
+      <c r="E5" s="10" t="inlineStr"/>
+      <c r="F5" s="10" t="inlineStr"/>
+      <c r="G5" s="10" t="inlineStr"/>
+      <c r="H5" s="11" t="inlineStr"/>
     </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6" ht="69" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>UT-M3-S2-02</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr"/>
+      <c r="F6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr"/>
+      <c r="H6" s="15" t="inlineStr"/>
     </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7" ht="55.5" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>UT-M3-S3-01</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="C7" s="10" t="inlineStr"/>
+      <c r="D7" s="10" t="inlineStr"/>
+      <c r="E7" s="10" t="inlineStr"/>
+      <c r="F7" s="10" t="inlineStr"/>
+      <c r="G7" s="10" t="inlineStr"/>
+      <c r="H7" s="11" t="inlineStr"/>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8" ht="39" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>UT-M3-S3-02</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="C8" s="14" t="inlineStr"/>
+      <c r="D8" s="14" t="inlineStr"/>
+      <c r="E8" s="14" t="inlineStr"/>
+      <c r="F8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr"/>
+      <c r="H8" s="15" t="inlineStr"/>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>UT-M3-S3-03</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr"/>
+      <c r="D9" s="18" t="inlineStr"/>
+      <c r="E9" s="18" t="inlineStr"/>
+      <c r="F9" s="18" t="inlineStr"/>
+      <c r="G9" s="18" t="inlineStr"/>
+      <c r="H9" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
test(M3): add Sprint 2 unit test evidence and fix controller test wiring
- Fill UT-M3-S2-01/02/03 rows in test evidence table (closeTopic scenarios)
- Add S2-screenshot.png showing mvn test BUILD SUCCESS (28 tests, 0 failures)
- Add missing @MockBean for TopicStatusService in ProjectTopicControllerStudentTest
  to fix ApplicationContext load failure introduced after Sprint 1 controller change
</commit_message>
<xml_diff>
--- a/test-evidence/M3-Cao-Yuhan/UT-M3-table.xlsx
+++ b/test-evidence/M3-Cao-Yuhan/UT-M3-table.xlsx
@@ -1276,7 +1276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="17.5663716814159" customWidth="1" min="1" max="1"/>
@@ -1464,12 +1464,36 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr"/>
-      <c r="D5" s="10" t="inlineStr"/>
-      <c r="E5" s="10" t="inlineStr"/>
-      <c r="F5" s="10" t="inlineStr"/>
-      <c r="G5" s="10" t="inlineStr"/>
-      <c r="H5" s="11" t="inlineStr"/>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>TopicStatusServiceImpl under test; topic (id=10) is in available status, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>closeTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Returns ProjectTopic with status = closed.</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Topic status changes to closed when closed by owner from available state.</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Returned topic has status = closed as asserted by assertEquals.</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="69" customHeight="1">
       <c r="A6" s="15" t="inlineStr">
@@ -1482,66 +1506,132 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr"/>
-      <c r="E6" s="14" t="inlineStr"/>
-      <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
-      <c r="H6" s="15" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Topic (id=10) is already in closed status, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>closeTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Throws IllegalStateException with message "Topic is already closed".</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Already-closed topic cannot be closed again; exception message is clear.</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>IllegalStateException thrown with expected message as asserted by assertThrows.</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="55.5" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>UT-M3-S3-01</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 3</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr"/>
-      <c r="D7" s="10" t="inlineStr"/>
-      <c r="E7" s="10" t="inlineStr"/>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="10" t="inlineStr"/>
-      <c r="H7" s="11" t="inlineStr"/>
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>UT-M3-S2-03</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Topic (id=10) is in unpublished status, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>closeTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Throws IllegalStateException with message "Only published topics can be closed".</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Unpublished topic cannot be closed; exception message is descriptive.</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>IllegalStateException thrown with expected message as asserted by assertThrows.</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="39" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>UT-M3-S3-02</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>UT-M3-S3-01</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr"/>
-      <c r="D8" s="14" t="inlineStr"/>
-      <c r="E8" s="14" t="inlineStr"/>
-      <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
-      <c r="H8" s="15" t="inlineStr"/>
+      <c r="C8" s="10" t="inlineStr"/>
+      <c r="D8" s="10" t="inlineStr"/>
+      <c r="E8" s="10" t="inlineStr"/>
+      <c r="F8" s="10" t="inlineStr"/>
+      <c r="G8" s="10" t="inlineStr"/>
+      <c r="H8" s="11" t="inlineStr"/>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>UT-M3-S3-02</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr"/>
+      <c r="D9" s="14" t="inlineStr"/>
+      <c r="E9" s="14" t="inlineStr"/>
+      <c r="F9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr"/>
+      <c r="H9" s="15" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>UT-M3-S3-03</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr"/>
-      <c r="D9" s="18" t="inlineStr"/>
-      <c r="E9" s="18" t="inlineStr"/>
-      <c r="F9" s="18" t="inlineStr"/>
-      <c r="G9" s="18" t="inlineStr"/>
-      <c r="H9" s="19" t="inlineStr"/>
+      <c r="C10" s="18" t="inlineStr"/>
+      <c r="D10" s="18" t="inlineStr"/>
+      <c r="E10" s="18" t="inlineStr"/>
+      <c r="F10" s="18" t="inlineStr"/>
+      <c r="G10" s="18" t="inlineStr"/>
+      <c r="H10" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
restore(M3): recover UT-M3-table.xlsx Sprint 1+2 content and formatting
File was overwritten by a binary merge conflict during Sprint 2 integration.
Restored from commit a2a3e28 which contains the filled Sprint 1 and Sprint 2 test evidence rows.
</commit_message>
<xml_diff>
--- a/test-evidence/M3-Cao-Yuhan/UT-M3-table.xlsx
+++ b/test-evidence/M3-Cao-Yuhan/UT-M3-table.xlsx
@@ -2,36 +2,194 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="20752" windowHeight="9555" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Tests" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="23">
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -40,16 +198,210 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -58,36 +410,513 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FFB2B2B2"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FFB2B2B2"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FFB2B2B2"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <dxfs count="7">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF08090C"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.8"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF08090C"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.8"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+  </dxfs>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="中色系标题行镶边行表格样式_6e22f3" count="7">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    </tableStyle>
+  </tableStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -438,7 +1267,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -448,168 +1276,362 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="17.5663716814159" customWidth="1" min="1" max="1"/>
+    <col width="11.7256637168142" customWidth="1" min="2" max="2"/>
+    <col width="50.3805309734513" customWidth="1" min="3" max="7"/>
+    <col width="16.3185840707965" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="22.5" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Test Name/ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Precondition (if any)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Output</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Expected</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Test process</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="65" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>UT-M3-S1-01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>ProjectTopicRepository and TopicStatusServiceImpl under test; topic (id=10) is unpublished, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>publishTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Returns ProjectTopic with status = available.</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Topic status changes to available when published by owner.</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Returned topic has status = available as asserted by assertEquals.</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="52" customHeight="1">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>UT-M3-S1-02</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Topic (id=10) is already in available status, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>publishTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Throws IllegalStateException with message "Only unpublished topics can be published".</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>Already-published topic cannot be published again; exception message is clear.</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>IllegalStateException thrown with expected message as asserted by assertThrows.</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="4" ht="73" customHeight="1">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>UT-M3-S1-03</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Topic (id=10) belongs to teacher (id=1), not teacher (id=99).</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>publishTopic(topicId=10, teacherId=99)</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Throws IllegalArgumentException with message "Topic not found or access denied".</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Topic not found or access denied for wrong teacher; ownership enforced.</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>IllegalArgumentException thrown with expected message as asserted by assertThrows.</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="67" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>UT-M3-S2-01</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>TopicStatusServiceImpl under test; topic (id=10) is in available status, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>closeTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Returns ProjectTopic with status = closed.</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Topic status changes to closed when closed by owner from available state.</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Returned topic has status = closed as asserted by assertEquals.</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6" ht="69" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>UT-M3-S2-02</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Topic (id=10) is already in closed status, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>closeTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Throws IllegalStateException with message "Topic is already closed".</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Already-closed topic cannot be closed again; exception message is clear.</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>IllegalStateException thrown with expected message as asserted by assertThrows.</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7" ht="55.5" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>UT-M3-S2-03</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Topic (id=10) is in unpublished status, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>closeTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Throws IllegalStateException with message "Only published topics can be closed".</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Unpublished topic cannot be closed; exception message is descriptive.</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>IllegalStateException thrown with expected message as asserted by assertThrows.</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="39" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>UT-M3-S3-01</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="C8" s="10" t="inlineStr"/>
+      <c r="D8" s="10" t="inlineStr"/>
+      <c r="E8" s="10" t="inlineStr"/>
+      <c r="F8" s="10" t="inlineStr"/>
+      <c r="G8" s="10" t="inlineStr"/>
+      <c r="H8" s="11" t="inlineStr"/>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>UT-M3-S3-02</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="C9" s="14" t="inlineStr"/>
+      <c r="D9" s="14" t="inlineStr"/>
+      <c r="E9" s="14" t="inlineStr"/>
+      <c r="F9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr"/>
+      <c r="H9" s="15" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>UT-M3-S3-03</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr"/>
+      <c r="D10" s="18" t="inlineStr"/>
+      <c r="E10" s="18" t="inlineStr"/>
+      <c r="F10" s="18" t="inlineStr"/>
+      <c r="G10" s="18" t="inlineStr"/>
+      <c r="H10" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
test(m3): add sprint 3 test evidence
</commit_message>
<xml_diff>
--- a/test-evidence/M3-Cao-Yuhan/UT-M3-table.xlsx
+++ b/test-evidence/M3-Cao-Yuhan/UT-M3-table.xlsx
@@ -1590,12 +1590,36 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr"/>
-      <c r="D8" s="10" t="inlineStr"/>
-      <c r="E8" s="10" t="inlineStr"/>
-      <c r="F8" s="10" t="inlineStr"/>
-      <c r="G8" s="10" t="inlineStr"/>
-      <c r="H8" s="11" t="inlineStr"/>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>TopicStatusServiceImpl under test; topic (id=10) is in closed status, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>archiveTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Returns ProjectTopic with status = archived.</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Topic status changes to archived when archived by owner from closed state.</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Returned topic has status = archived as asserted by assertEquals.</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="15" t="inlineStr">
@@ -1608,14 +1632,38 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr"/>
-      <c r="D9" s="14" t="inlineStr"/>
-      <c r="E9" s="14" t="inlineStr"/>
-      <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
-      <c r="H9" s="15" t="inlineStr"/>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Topic (id=10) is already in archived status, owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>archiveTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Throws IllegalStateException with message "Topic is already archived".</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>Already-archived topic cannot be archived again; exception message is clear.</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>IllegalStateException thrown with expected message as asserted by assertThrows.</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
-    <row r="10">
+    <row r="10" ht="70" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
         <is>
           <t>UT-M3-S3-03</t>
@@ -1626,12 +1674,36 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr"/>
-      <c r="D10" s="18" t="inlineStr"/>
-      <c r="E10" s="18" t="inlineStr"/>
-      <c r="F10" s="18" t="inlineStr"/>
-      <c r="G10" s="18" t="inlineStr"/>
-      <c r="H10" s="19" t="inlineStr"/>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Topic (id=10) is in available status (representing any non-closed state), owned by teacher (id=1).</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>archiveTopic(topicId=10, teacherId=1)</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Throws IllegalStateException with message "Topic must be closed before it can be archived".</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Topic in non-closed state cannot be archived; only closed topics are eligible.</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>IllegalStateException thrown with expected message as asserted by assertThrows.</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>